<commit_message>
added safe files to .gitignore
</commit_message>
<xml_diff>
--- a/data/allopathic_medicines.xlsx
+++ b/data/allopathic_medicines.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F51"/>
+  <dimension ref="A1:F52"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -2048,6 +2048,38 @@
         </is>
       </c>
     </row>
+    <row r="52">
+      <c r="A52" t="inlineStr">
+        <is>
+          <t>Varicose-vein-type condition</t>
+        </is>
+      </c>
+      <c r="B52" t="inlineStr">
+        <is>
+          <t>Micronized Purified Flavonoid Fraction (MPFF / Daflon), Horse Chestnut Extract</t>
+        </is>
+      </c>
+      <c r="C52" t="inlineStr">
+        <is>
+          <t>MPFF 500mg: 1 tablet twice daily with meals</t>
+        </is>
+      </c>
+      <c r="D52" t="inlineStr">
+        <is>
+          <t>2-3 months as advised by vascular specialist</t>
+        </is>
+      </c>
+      <c r="E52" t="inlineStr">
+        <is>
+          <t>High fiber diet, flavonoids (berries, citrus), low sodium to reduce fluid retention</t>
+        </is>
+      </c>
+      <c r="F52" t="inlineStr">
+        <is>
+          <t>Graduated compression stockings (Class 2), elevate legs 15-20 min daily, avoid prolonged standing</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>